<commit_message>
feat: added the user overtime detail in excel export
</commit_message>
<xml_diff>
--- a/data/sheet.xlsx
+++ b/data/sheet.xlsx
@@ -12,15 +12,81 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3" uniqueCount="3">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="25">
   <si>
     <t>OVERTIME APPROVAL SHEET</t>
   </si>
   <si>
-    <t>Employee Name: Kamal Giri</t>
+    <t>Employee Name: Apurba Rajyashree Thapa</t>
   </si>
   <si>
     <t>Employee Department: Java</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Project or description of work overtime </t>
+  </si>
+  <si>
+    <t>1.Gym Management System</t>
+  </si>
+  <si>
+    <t>2.Over Time System</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Date </t>
+  </si>
+  <si>
+    <t>Day</t>
+  </si>
+  <si>
+    <t>From(Time)</t>
+  </si>
+  <si>
+    <t>To(Time)</t>
+  </si>
+  <si>
+    <t>Total Hour</t>
+  </si>
+  <si>
+    <t>2023-04-25</t>
+  </si>
+  <si>
+    <t>TUESDAY</t>
+  </si>
+  <si>
+    <t>07:00</t>
+  </si>
+  <si>
+    <t>09:00</t>
+  </si>
+  <si>
+    <t>09:40</t>
+  </si>
+  <si>
+    <t>00:40</t>
+  </si>
+  <si>
+    <t>12:04</t>
+  </si>
+  <si>
+    <t>14:04</t>
+  </si>
+  <si>
+    <t>16:48</t>
+  </si>
+  <si>
+    <t>19:48</t>
+  </si>
+  <si>
+    <t>2023-04-27</t>
+  </si>
+  <si>
+    <t>THURSDAY</t>
+  </si>
+  <si>
+    <t>15:42</t>
+  </si>
+  <si>
+    <t>18:42</t>
   </si>
 </sst>
 </file>
@@ -28,13 +94,17 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <sz val="11.0"/>
       <color indexed="8"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="12.0"/>
     </font>
   </fonts>
   <fills count="2">
@@ -57,19 +127,30 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyAlignment="true" applyFont="true">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="true">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="true"/>
   </cellXfs>
 </styleSheet>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="B2:B5"/>
+  <dimension ref="B2:F14"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
+  <cols>
+    <col min="2" max="2" width="12.3359375" customWidth="true" bestFit="true"/>
+    <col min="3" max="3" width="10.15234375" customWidth="true" bestFit="true"/>
+    <col min="4" max="4" width="12.54296875" customWidth="true" bestFit="true"/>
+    <col min="5" max="5" width="9.85546875" customWidth="true" bestFit="true"/>
+    <col min="6" max="6" width="11.4765625" customWidth="true" bestFit="true"/>
+  </cols>
   <sheetData>
     <row r="2">
       <c r="B2" t="s" s="1">
@@ -86,11 +167,129 @@
         <v>2</v>
       </c>
     </row>
+    <row r="6">
+      <c r="B6" t="s" s="2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="B7" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="B8" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="B9" t="s" s="1">
+        <v>6</v>
+      </c>
+      <c r="C9" t="s" s="1">
+        <v>7</v>
+      </c>
+      <c r="D9" t="s" s="1">
+        <v>8</v>
+      </c>
+      <c r="E9" t="s" s="1">
+        <v>9</v>
+      </c>
+      <c r="F9" t="s" s="1">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="B10" t="s" s="3">
+        <v>11</v>
+      </c>
+      <c r="C10" t="s" s="3">
+        <v>12</v>
+      </c>
+      <c r="D10" t="s" s="3">
+        <v>13</v>
+      </c>
+      <c r="E10" t="s" s="3">
+        <v>14</v>
+      </c>
+      <c r="F10" t="n" s="3">
+        <v>120.0</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="B11" t="s" s="3">
+        <v>11</v>
+      </c>
+      <c r="C11" t="s" s="3">
+        <v>12</v>
+      </c>
+      <c r="D11" t="s" s="3">
+        <v>15</v>
+      </c>
+      <c r="E11" t="s" s="3">
+        <v>16</v>
+      </c>
+      <c r="F11" t="n" s="3">
+        <v>-540.0</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="B12" t="s" s="3">
+        <v>11</v>
+      </c>
+      <c r="C12" t="s" s="3">
+        <v>12</v>
+      </c>
+      <c r="D12" t="s" s="3">
+        <v>17</v>
+      </c>
+      <c r="E12" t="s" s="3">
+        <v>18</v>
+      </c>
+      <c r="F12" t="n" s="3">
+        <v>120.0</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="B13" t="s" s="3">
+        <v>11</v>
+      </c>
+      <c r="C13" t="s" s="3">
+        <v>12</v>
+      </c>
+      <c r="D13" t="s" s="3">
+        <v>19</v>
+      </c>
+      <c r="E13" t="s" s="3">
+        <v>20</v>
+      </c>
+      <c r="F13" t="n" s="3">
+        <v>180.0</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="B14" t="s" s="3">
+        <v>21</v>
+      </c>
+      <c r="C14" t="s" s="3">
+        <v>22</v>
+      </c>
+      <c r="D14" t="s" s="3">
+        <v>23</v>
+      </c>
+      <c r="E14" t="s" s="3">
+        <v>24</v>
+      </c>
+      <c r="F14" t="n" s="3">
+        <v>180.0</v>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="3">
+  <mergeCells count="4">
     <mergeCell ref="B2:F3"/>
     <mergeCell ref="B4:F4"/>
     <mergeCell ref="B5:F5"/>
+    <mergeCell ref="B6:F8"/>
   </mergeCells>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>

</xml_diff>

<commit_message>
fix: completed the excel sheet format
</commit_message>
<xml_diff>
--- a/data/sheet.xlsx
+++ b/data/sheet.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="25">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="32">
   <si>
     <t>OVERTIME APPROVAL SHEET</t>
   </si>
@@ -59,12 +59,6 @@
     <t>09:00</t>
   </si>
   <si>
-    <t>09:40</t>
-  </si>
-  <si>
-    <t>00:40</t>
-  </si>
-  <si>
     <t>12:04</t>
   </si>
   <si>
@@ -87,6 +81,34 @@
   </si>
   <si>
     <t>18:42</t>
+  </si>
+  <si>
+    <t xml:space="preserve">=SUM(F15:F12)
+</t>
+  </si>
+  <si>
+    <t>I certify that this is a true and correct claim of overtime incurred by me on the above dates.</t>
+  </si>
+  <si>
+    <t>_______________________</t>
+  </si>
+  <si>
+    <t>Employee's Signature</t>
+  </si>
+  <si>
+    <t>Date: 2023-05-02</t>
+  </si>
+  <si>
+    <t>I certify that this is a true and correct claim of overtime incurred by the above employee on the above dates. Therefore, I recommend payment for the above overtime.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Supervisor’s signature </t>
+  </si>
+  <si>
+    <t xml:space="preserve">HR Approval </t>
+  </si>
+  <si>
+    <t xml:space="preserve">HR Representative </t>
   </si>
 </sst>
 </file>
@@ -142,10 +164,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="B2:F14"/>
+  <dimension ref="B2:F31"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
-    <col min="2" max="2" width="12.3359375" customWidth="true" bestFit="true"/>
+    <col min="2" max="2" width="36.76953125" customWidth="true" bestFit="true"/>
     <col min="3" max="3" width="10.15234375" customWidth="true" bestFit="true"/>
     <col min="4" max="4" width="12.54296875" customWidth="true" bestFit="true"/>
     <col min="5" max="5" width="9.85546875" customWidth="true" bestFit="true"/>
@@ -167,70 +189,38 @@
         <v>2</v>
       </c>
     </row>
-    <row r="6">
-      <c r="B6" t="s" s="2">
+    <row r="6"/>
+    <row r="7">
+      <c r="B7" t="s" s="2">
         <v>3</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="B7" t="s">
-        <v>4</v>
       </c>
     </row>
     <row r="8">
       <c r="B8" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="B9" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="9">
-      <c r="B9" t="s" s="1">
+    <row r="10"/>
+    <row r="11">
+      <c r="B11" t="s" s="1">
         <v>6</v>
       </c>
-      <c r="C9" t="s" s="1">
+      <c r="C11" t="s" s="1">
         <v>7</v>
       </c>
-      <c r="D9" t="s" s="1">
+      <c r="D11" t="s" s="1">
         <v>8</v>
       </c>
-      <c r="E9" t="s" s="1">
+      <c r="E11" t="s" s="1">
         <v>9</v>
       </c>
-      <c r="F9" t="s" s="1">
+      <c r="F11" t="s" s="1">
         <v>10</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="B10" t="s" s="3">
-        <v>11</v>
-      </c>
-      <c r="C10" t="s" s="3">
-        <v>12</v>
-      </c>
-      <c r="D10" t="s" s="3">
-        <v>13</v>
-      </c>
-      <c r="E10" t="s" s="3">
-        <v>14</v>
-      </c>
-      <c r="F10" t="n" s="3">
-        <v>120.0</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="B11" t="s" s="3">
-        <v>11</v>
-      </c>
-      <c r="C11" t="s" s="3">
-        <v>12</v>
-      </c>
-      <c r="D11" t="s" s="3">
-        <v>15</v>
-      </c>
-      <c r="E11" t="s" s="3">
-        <v>16</v>
-      </c>
-      <c r="F11" t="n" s="3">
-        <v>-540.0</v>
       </c>
     </row>
     <row r="12">
@@ -241,13 +231,13 @@
         <v>12</v>
       </c>
       <c r="D12" t="s" s="3">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="E12" t="s" s="3">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="F12" t="n" s="3">
-        <v>120.0</v>
+        <v>2.0</v>
       </c>
     </row>
     <row r="13">
@@ -258,38 +248,128 @@
         <v>12</v>
       </c>
       <c r="D13" t="s" s="3">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="E13" t="s" s="3">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="F13" t="n" s="3">
-        <v>180.0</v>
+        <v>2.0</v>
       </c>
     </row>
     <row r="14">
       <c r="B14" t="s" s="3">
+        <v>11</v>
+      </c>
+      <c r="C14" t="s" s="3">
+        <v>12</v>
+      </c>
+      <c r="D14" t="s" s="3">
+        <v>17</v>
+      </c>
+      <c r="E14" t="s" s="3">
+        <v>18</v>
+      </c>
+      <c r="F14" t="n" s="3">
+        <v>3.0</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="B15" t="s" s="3">
+        <v>19</v>
+      </c>
+      <c r="C15" t="s" s="3">
+        <v>20</v>
+      </c>
+      <c r="D15" t="s" s="3">
         <v>21</v>
       </c>
-      <c r="C14" t="s" s="3">
+      <c r="E15" t="s" s="3">
         <v>22</v>
       </c>
-      <c r="D14" t="s" s="3">
+      <c r="F15" t="n" s="3">
+        <v>3.0</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="B16" t="s" s="1">
+        <v>10</v>
+      </c>
+      <c r="F16" t="s">
         <v>23</v>
       </c>
-      <c r="E14" t="s" s="3">
+    </row>
+    <row r="17"/>
+    <row r="18">
+      <c r="B18" t="s">
         <v>24</v>
       </c>
-      <c r="F14" t="n" s="3">
-        <v>180.0</v>
+    </row>
+    <row r="20">
+      <c r="B20" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="B21" t="s">
+        <v>26</v>
+      </c>
+      <c r="E21" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="B23" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="B25" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="B26" t="s">
+        <v>29</v>
+      </c>
+      <c r="E26" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="B28" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="B30" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="B31" t="s">
+        <v>31</v>
+      </c>
+      <c r="E31" t="s">
+        <v>27</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="4">
+  <mergeCells count="14">
     <mergeCell ref="B2:F3"/>
     <mergeCell ref="B4:F4"/>
     <mergeCell ref="B5:F5"/>
-    <mergeCell ref="B6:F8"/>
+    <mergeCell ref="B16:E16"/>
+    <mergeCell ref="B18:F18"/>
+    <mergeCell ref="B19:F19"/>
+    <mergeCell ref="B20:F20"/>
+    <mergeCell ref="B22:F22"/>
+    <mergeCell ref="B23:N23"/>
+    <mergeCell ref="B24:N24"/>
+    <mergeCell ref="B25:F25"/>
+    <mergeCell ref="B27:F27"/>
+    <mergeCell ref="B29:F29"/>
+    <mergeCell ref="B30:F30"/>
   </mergeCells>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>

</xml_diff>